<commit_message>
Turn Lou into a multi-playbook demo
Make the Pioneer dataset materialize into runtime playbooks, refresh the Company Brain around playbook-first memory, and harden launch/smoke checks around the generated data.

Also document the 50-playbook Pioneer matrix flow and make the matrix generator top up missing playbook specs instead of failing when Pioneer returns a short batch.
</commit_message>
<xml_diff>
--- a/demo-data/siemens-mutual-nda-playbook.xlsx
+++ b/demo-data/siemens-mutual-nda-playbook.xlsx
@@ -456,370 +456,370 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NDA Scope</t>
+          <t>NDA Confidentiality Scope</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Confidentiality limited to specific defined information.</t>
+          <t>Confidential information includes all non-public data, including internal strategies and customer lists.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Confidentiality limited to information explicitly identified in the agreement.</t>
+          <t>Confidential information includes all non-public data, excluding customer lists.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Confidentiality limited to information provided in writing.</t>
+          <t>Confidential information includes all non-public data, excluding internal strategies.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Confidentiality limited to information shared during meetings.</t>
+          <t>Confidential information includes all non-public data, excluding customer lists and internal strategies.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Confidentiality includes all information exchanged during discussions.</t>
+          <t>Confidential information includes all non-public data, including internal strategies, customer lists, and financial records.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Confidentiality includes all information, including non-disclosure of sensitive internal processes.</t>
+          <t>Confidential information includes all non-public data, including internal strategies, customer lists, financial records, and proprietary algorithms.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SaaS Termination Notice Period</t>
+          <t>SaaS Data Processing</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>30-day written notice period with automatic renewal unless terminated.</t>
+          <t>Data processing is limited to the scope of the service provided and does not include third-party sharing without consent.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>30-day written notice period with automatic renewal unless terminated.</t>
+          <t>Data processing is limited to the scope of the service provided and does not include third-party sharing without explicit consent.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>15-day written notice period with automatic renewal unless terminated.</t>
+          <t>Data processing is limited to the scope of the service provided and does not include third-party sharing.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>7-day written notice period with automatic renewal unless terminated.</t>
+          <t>Data processing is limited to the scope of the service provided.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>No notice period required for termination.</t>
+          <t>Data processing includes all data handling activities, including third-party sharing without consent.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Termination without notice or penalty.</t>
+          <t>Data processing includes all data handling activities, including third-party sharing without consent and without prior notice.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Data Processing Compliance</t>
+          <t>AI Vendor Terms</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Compliance with GDPR and CCPA standards.</t>
+          <t>AI model training includes only customer data provided for the purpose of the service.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Compliance with GDPR and other applicable data protection laws.</t>
+          <t>AI model training includes only customer data provided for the purpose of the service, excluding sensitive personal information.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Compliance with minimum data protection standards.</t>
+          <t>AI model training includes only customer data provided for the purpose of the service, excluding personally identifiable information.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Compliance with basic data protection requirements.</t>
+          <t>AI model training includes only customer data provided for the purpose of the service, excluding non-sensitive data.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>No data protection obligations imposed on the vendor.</t>
+          <t>AI model training includes all customer data, including sensitive personal information.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Data processing without any legal compliance requirements.</t>
+          <t>AI model training includes all customer data, including sensitive personal information, and may be used for unrelated purposes.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Security Incident Response</t>
+          <t>IP Ownership in SaaS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>72-hour notification of security incidents with full disclosure.</t>
+          <t>All IP developed during the engagement is owned by the client, including source code and documentation.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>48-hour notification of security incidents with partial disclosure.</t>
+          <t>All IP developed during the engagement is owned by the client, including source code, but not documentation.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>24-hour notification of security incidents with limited disclosure.</t>
+          <t>All IP developed during the engagement is owned by the client, including documentation, but not source code.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Notification within 12 hours with no disclosure required.</t>
+          <t>All IP developed during the engagement is owned by the client, excluding any IP developed by the vendor.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>No obligation to notify of security incidents.</t>
+          <t>All IP developed during the engagement is owned by the vendor, including source code and documentation.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>No obligation to notify or remediate security incidents.</t>
+          <t>All IP developed during the engagement is owned by the vendor, including source code, documentation, and any derivative works.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>IP Ownership</t>
+          <t>Professional Services Contract Term</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>All IP developed during the engagement belongs to the client.</t>
+          <t>Term is for a fixed period of 12 months with an option to renew for an additional 12 months.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>IP developed during the engagement is owned by the client unless otherwise agreed.</t>
+          <t>Term is for a fixed period of 12 months with an option to renew for an additional 6 months.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>IP developed during the engagement is owned by the client, with exceptions for third-party IP.</t>
+          <t>Term is for a fixed period of 12 months with an option to renew for an additional 3 months.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>IP developed during the engagement is owned by the client, with limited exceptions.</t>
+          <t>Term is for a fixed period of 12 months with no renewal option.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>IP ownership is not specified or transferred.</t>
+          <t>Term is for a fixed period of 12 months with no renewal option and no notice period.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>IP ownership remains with the vendor.</t>
+          <t>Term is for a fixed period of 12 months with no renewal option, no notice period, and no right to terminate.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Procurement Terms</t>
+          <t>Enterprise Software Security Requirements</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fixed-price contract with clear deliverables and payment milestones.</t>
+          <t>All software must meet ISO 27001 security standards and undergo annual penetration testing.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fixed-price contract with clear deliverables and payment milestones.</t>
+          <t>All software must meet ISO 27001 security standards and undergo bi-annual penetration testing.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Fixed-price contract with clear deliverables and no payment milestones.</t>
+          <t>All software must meet ISO 27001 security standards and undergo annual security audits.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Fixed-price contract with limited deliverables and no payment milestones.</t>
+          <t>All software must meet ISO 27001 security standards.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>No fixed-price terms or deliverables defined.</t>
+          <t>All software must meet ISO 27001 security standards and undergo quarterly security audits.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>No contract terms defined or agreed upon.</t>
+          <t>All software must meet ISO 27001 security standards and undergo no security audits or testing.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AI Vendor Terms</t>
+          <t>Data Processing Agreement Compliance</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AI models are trained on non-sensitive, anonymized data only.</t>
+          <t>Data processing complies with GDPR and CCPA, with regular audits and data breach notifications.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AI models are trained on non-sensitive data with limited anonymization.</t>
+          <t>Data processing complies with GDPR and CCPA, with regular audits.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>AI models are trained on non-sensitive data with minimal anonymization.</t>
+          <t>Data processing complies with GDPR and CCPA, with data breach notifications.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AI models are trained on non-sensitive data with no anonymization.</t>
+          <t>Data processing complies with GDPR and CCPA.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AI models are trained on any data without restrictions.</t>
+          <t>Data processing complies with GDPR and CCPA, but no audits or breach notifications are required.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>AI models are trained on any data, including sensitive and personal information.</t>
+          <t>Data processing complies with GDPR and CCPA, but no audits, breach notifications, or data protection impact assessments are required.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Professional Services Scope</t>
+          <t>Procurement Contract Term Limits</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Scope defined in detail with deliverables and timelines.</t>
+          <t>Term is limited to the duration of the project with a 30-day termination notice period.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Scope defined in detail with deliverables but no timelines.</t>
+          <t>Term is limited to the duration of the project with a 15-day termination notice period.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Scope defined with general deliverables and timelines.</t>
+          <t>Term is limited to the duration of the project with a 7-day termination notice period.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Scope defined with limited deliverables and timelines.</t>
+          <t>Term is limited to the duration of the project with no termination notice period.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Scope not defined or agreed upon.</t>
+          <t>Term is limited to the duration of the project with no termination notice period and no right to terminate.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>No defined scope or deliverables.</t>
+          <t>Term is limited to the duration of the project with no termination notice period, no right to terminate, and no exit clauses.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Enterprise Software Licensing</t>
+          <t>Security Incident Response Plan</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Licensing based on user count with annual renewal options.</t>
+          <t>The vendor must provide a 24/7 security incident response team and notify the client within 2 hours of a breach.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Licensing based on user count with annual renewal options.</t>
+          <t>The vendor must provide a 24/7 security incident response team and notify the client within 4 hours of a breach.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Licensing based on user count with no renewal options.</t>
+          <t>The vendor must provide a 24/7 security incident response team and notify the client within 8 hours of a breach.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Licensing based on user count with limited renewal options.</t>
+          <t>The vendor must provide a 24/7 security incident response team and notify the client within 12 hours of a breach.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Licensing based on usage with no user count restrictions.</t>
+          <t>The vendor must provide a 24/7 security incident response team and notify the client within 24 hours of a breach.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Licensing based on usage with no user count or renewal options.</t>
+          <t>The vendor must provide a 24/7 security incident response team and notify the client within 72 hours of a breach.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Data Residency Requirements</t>
+          <t>IP Licensing in AI Models</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Data stored within the EU and subject to EU data protection laws.</t>
+          <t>Licensing includes all AI models, training data, and associated algorithms for commercial use.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Data stored within the EU or other specified regions.</t>
+          <t>Licensing includes all AI models and associated algorithms for commercial use, excluding training data.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Data stored within the EU or other regions with minimal restrictions.</t>
+          <t>Licensing includes all AI models for commercial use, excluding training data and associated algorithms.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Data stored within the EU or other regions with no restrictions.</t>
+          <t>Licensing includes all AI models for commercial use, excluding training data, associated algorithms, and derivative works.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Data stored outside of the EU with no restrictions.</t>
+          <t>Licensing includes all AI models, training data, and associated algorithms for non-commercial use only.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Data stored anywhere without restrictions.</t>
+          <t>Licensing includes all AI models, training data, and associated algorithms for non-commercial use only and no commercial use is permitted.</t>
         </is>
       </c>
     </row>
@@ -831,735 +831,735 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Confidentiality obligations apply to all disclosed information, including trade secrets, and remain in effect for 5 years.</t>
+          <t>Both parties agree to mutual non-disclosure of all confidential information exchanged during negotiations.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Confidentiality obligations apply to all disclosed information, including trade secrets, and remain in effect for 3 years.</t>
+          <t>Confidentiality is limited to information disclosed by the other party.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Confidentiality obligations apply to all disclosed information, but the duration is negotiable.</t>
+          <t>Confidentiality applies only to information disclosed in writing.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Confidentiality obligations apply only to information explicitly marked as confidential.</t>
+          <t>Confidentiality is limited to information disclosed in the course of business.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Confidentiality obligations do not apply to any information disclosed during the term of the agreement.</t>
+          <t>Confidentiality must extend to all information exchanged, including verbal communications.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Confidentiality obligations do not apply to any information and the other party is not bound by any duty of confidentiality.</t>
+          <t>Disclosure of any information is permitted without restriction.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SaaS Data Ownership</t>
+          <t>SaaS Service Level Agreement</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Customer retains ownership of all data processed by the SaaS platform, including derivative data.</t>
+          <t>Service level objectives are defined with clear performance metrics and penalties for non-compliance.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Customer retains ownership of all data processed by the SaaS platform, including derivative data, but the provider may retain copies for backup purposes.</t>
+          <t>Service level objectives are defined with performance metrics but no penalties.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Customer retains ownership of all data processed by the SaaS platform, but the provider may retain copies for backup purposes.</t>
+          <t>Service level objectives are outlined but not quantified.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Customer retains ownership of all data processed by the SaaS platform, but the provider may retain copies for operational use.</t>
+          <t>Service level expectations are general and not specified.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Customer does not retain ownership of any data processed by the SaaS platform.</t>
+          <t>Performance metrics must include penalties for non-compliance and service credits.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Customer does not retain ownership of any data and the provider owns all data processed through the platform.</t>
+          <t>No service level objectives or performance metrics are required.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Data Processing Agreement Scope</t>
+          <t>Data Processing Agreement</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>The agreement applies to all data processing activities, including third-party data transfers and subprocessing.</t>
+          <t>Data processing is limited to the specific purposes outlined in the agreement.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>The agreement applies to all data processing activities, including third-party data transfers, but not subprocessing.</t>
+          <t>Data processing is limited to the purposes reasonably necessary for the service provided.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>The agreement applies to all data processing activities, but subprocessing is subject to additional approval.</t>
+          <t>Data processing is permitted for any purpose related to the service.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>The agreement applies to all data processing activities, but subprocessing is not explicitly covered.</t>
+          <t>Data processing is allowed without restriction.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>The agreement does not apply to any data processing activities outside of the initial scope.</t>
+          <t>Data processing must include explicit consent from data subjects for all uses.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The agreement does not apply to any data processing activities and the provider is not bound by any obligations.</t>
+          <t>Data can be processed for any purpose without consent or restriction.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Security Incident Response</t>
+          <t>Security Compliance Requirements</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>The provider must notify the customer of any security incident within 24 hours and provide a detailed incident report within 7 days.</t>
+          <t>The service provider must comply with ISO 27001 and SOC 2 standards.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>The provider must notify the customer of any security incident within 48 hours and provide a detailed incident report within 14 days.</t>
+          <t>The service provider must comply with at least one of ISO 27001 or SOC 2 standards.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>The provider must notify the customer of any security incident within 72 hours and provide a detailed incident report within 30 days.</t>
+          <t>The service provider must implement basic security controls as outlined in the agreement.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>The provider must notify the customer of any security incident within 7 days and provide a detailed incident report within 60 days.</t>
+          <t>The service provider must provide a general security policy.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>The provider is not required to notify the customer of any security incidents.</t>
+          <t>The service provider must provide third-party audit reports for all security measures.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>The provider is not required to notify the customer of any security incidents and is not bound by any incident response obligations.</t>
+          <t>No security requirements or audits are required.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IP Assignment in Procurement</t>
+          <t>IP Ownership in AI Vendor Terms</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>All IP developed by the vendor during the performance of the contract is assigned to the customer.</t>
+          <t>All intellectual property developed during the engagement is owned by the client.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>All IP developed by the vendor during the performance of the contract is assigned to the customer, but the vendor retains rights to use the IP for its own purposes.</t>
+          <t>IP developed during the engagement is owned by the client unless otherwise agreed.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>All IP developed by the vendor during the performance of the contract is assigned to the customer, but the vendor may retain non-exclusive rights for internal use.</t>
+          <t>IP developed during the engagement is jointly owned by both parties.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>All IP developed by the vendor during the performance of the contract is assigned to the customer, but the vendor may retain rights to use the IP for its own purposes.</t>
+          <t>IP developed during the engagement is owned by the vendor unless specified otherwise.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>The vendor is not required to assign any IP developed during the performance of the contract.</t>
+          <t>IP ownership must be determined by a third-party IP audit.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>The vendor is not required to assign any IP and retains all rights to any IP developed during the performance of the contract.</t>
+          <t>IP ownership is not specified and defaults to vendor ownership.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AI Vendor Model Usage Rights</t>
+          <t>Professional Services Termination Clause</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>The customer has exclusive rights to use the AI model for the agreed purpose, and the vendor may not use the model for any other purpose.</t>
+          <t>Either party may terminate the agreement with 30 days' written notice.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The customer has exclusive rights to use the AI model for the agreed purpose, but the vendor may use the model for research and development purposes.</t>
+          <t>Either party may terminate the agreement with 15 days' written notice.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>The customer has exclusive rights to use the AI model for the agreed purpose, but the vendor may use the model for non-commercial purposes.</t>
+          <t>Either party may terminate the agreement with 7 days' written notice.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>The customer has exclusive rights to use the AI model for the agreed purpose, but the vendor may use the model for internal testing.</t>
+          <t>Either party may terminate the agreement without notice.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>The customer does not have exclusive rights to use the AI model and the vendor may use the model for any purpose.</t>
+          <t>Termination requires a court order or mutual agreement.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>The customer does not have exclusive rights to use the AI model and the vendor may use the model for any purpose, including commercial use.</t>
+          <t>Termination is not permitted under any circumstances.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Professional Services Contract Term</t>
+          <t>Enterprise Software Customization Rights</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>The contract term is for 12 months with automatic renewal unless terminated 60 days in advance.</t>
+          <t>The client retains full rights to customize the software as needed.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>The contract term is for 12 months with automatic renewal unless terminated 90 days in advance.</t>
+          <t>The client has limited rights to customize the software with vendor approval.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>The contract term is for 12 months with automatic renewal unless terminated 180 days in advance.</t>
+          <t>The client may request customizations but must pay additional fees.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>The contract term is for 12 months with automatic renewal unless terminated 365 days in advance.</t>
+          <t>Customizations are not permitted without significant approval processes.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>The contract term is for 12 months with no automatic renewal and no termination notice required.</t>
+          <t>Customization rights are limited to pre-approved features only.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>The contract term is for 12 months with no automatic renewal and the customer may terminate the contract at any time without notice.</t>
+          <t>Customization is not allowed under any circumstances.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Enterprise Software Customization Rights</t>
+          <t>Procurement Contract Payment Terms</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>The customer has the right to customize the software to meet its specific business needs, with no restrictions on the scope of customization.</t>
+          <t>Payment is due within 15 days of receipt of invoice.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>The customer has the right to customize the software to meet its specific business needs, but the vendor may impose reasonable restrictions on the scope of customization.</t>
+          <t>Payment is due within 30 days of receipt of invoice.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>The customer has the right to customize the software to meet its specific business needs, but the vendor may require approval for major customizations.</t>
+          <t>Payment is due within 60 days of receipt of invoice.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>The customer has the right to customize the software to meet its specific business needs, but the vendor may require a fee for customizations.</t>
+          <t>Payment terms are flexible and not specified.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>The customer does not have the right to customize the software and the vendor may impose restrictions on any customizations.</t>
+          <t>Payment must be made within 7 days of receipt of invoice with interest for late payments.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>The customer does not have the right to customize the software and the vendor may impose restrictions on all customizations, including internal use.</t>
+          <t>No payment terms are specified and payment is due upon delivery.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Data Breach Notification Requirements</t>
+          <t>AI Vendor Data Access Controls</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>The vendor must notify the customer of any data breach within 24 hours and provide a detailed report within 7 days.</t>
+          <t>The vendor must implement strict access controls to protect client data.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>The vendor must notify the customer of any data breach within 48 hours and provide a detailed report within 14 days.</t>
+          <t>The vendor must implement basic access controls to protect client data.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>The vendor must notify the customer of any data breach within 72 hours and provide a detailed report within 30 days.</t>
+          <t>The vendor must provide access controls as outlined in the agreement.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>The vendor must notify the customer of any data breach within 7 days and provide a detailed report within 60 days.</t>
+          <t>The vendor may access data as needed without restrictions.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>The vendor is not required to notify the customer of any data breaches.</t>
+          <t>The vendor must provide a detailed access control policy and audit logs.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>The vendor is not required to notify the customer of any data breaches and is not bound by any breach notification obligations.</t>
+          <t>The vendor has unrestricted access to all client data.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Third-Party Access to Customer Data</t>
+          <t>Data Breach Notification Requirements</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>The vendor may not allow any third-party access to customer data without the customer's prior written consent.</t>
+          <t>The vendor must notify the client within 24 hours of discovering a data breach.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>The vendor may not allow any third-party access to customer data without the customer's prior written consent, but may share data with service providers for operational purposes.</t>
+          <t>The vendor must notify the client within 48 hours of discovering a data breach.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>The vendor may not allow any third-party access to customer data without the customer's prior written consent, but may share data with service providers for operational purposes with limited access.</t>
+          <t>The vendor must notify the client within 72 hours of discovering a data breach.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>The vendor may not allow any third-party access to customer data without the customer's prior written consent, but may share data with service providers for operational purposes with limited access and oversight.</t>
+          <t>The vendor must notify the client within 7 days of discovering a data breach.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>The vendor may allow any third-party access to customer data without the customer's consent.</t>
+          <t>The vendor must provide a detailed breach report within 24 hours.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>The vendor may allow any third-party access to customer data without the customer's consent and is not bound by any restrictions on data sharing.</t>
+          <t>The vendor is not required to notify the client of any data breaches.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NDA Mutual Non-Disclosure</t>
+          <t>NDA Scope</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Both parties agree to mutual non-disclosure of all confidential information exchanged during negotiations.</t>
+          <t>Confidentiality limited to proprietary information and trade secrets.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Confidentiality applies only to the disclosing party's information.</t>
+          <t>Confidentiality limited to information explicitly identified in the agreement.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Confidentiality is limited to information shared in written form.</t>
+          <t>Confidentiality limited to information exchanged during the term of the agreement.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Confidentiality applies only to information shared in the presence of both parties.</t>
+          <t>Confidentiality limited to information relevant to the negotiation.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Confidentiality does not apply to information shared by the other party.</t>
+          <t>Confidentiality includes all information exchanged regardless of relevance.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>No confidentiality obligations apply to either party.</t>
+          <t>Confidentiality includes all information, including non-proprietary and public information.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SaaS Data Processing</t>
+          <t>SaaS Data Ownership</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>The service provider must comply with all applicable data protection laws and regulations.</t>
+          <t>Customer retains ownership of all data processed through the service.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>The service provider will comply with data protection laws in the jurisdiction where the data is processed.</t>
+          <t>Customer retains ownership of data processed through the service, excluding data generated by the service.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>The service provider will comply with data protection laws in the jurisdiction of the client.</t>
+          <t>Customer retains ownership of data processed through the service, excluding data subject to third-party rights.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>The service provider will comply with data protection laws in the jurisdiction of the service provider.</t>
+          <t>Customer retains ownership of data processed through the service, excluding data subject to service provider's intellectual property.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>The service provider is not required to comply with data protection laws.</t>
+          <t>Service provider retains ownership of all data processed through the service.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>No data protection obligations apply to the service provider.</t>
+          <t>Service provider retains ownership of all data, including data generated by the customer.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AI Vendor Terms Model Ownership</t>
+          <t>Data Processing Agreement</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>The AI model developed by the vendor is owned by the client upon payment of the final milestone.</t>
+          <t>Processor is prohibited from using data for purposes other than those specified in the agreement.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>The AI model is owned by the client upon completion of the project.</t>
+          <t>Processor is prohibited from using data for purposes other than those specified in the agreement, excluding incidental use for system maintenance.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>The AI model is owned by the client upon acceptance of deliverables.</t>
+          <t>Processor is prohibited from using data for purposes other than those specified in the agreement, excluding use for legal compliance.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>The AI model is owned by the client upon receipt of the final deliverable.</t>
+          <t>Processor is prohibited from using data for purposes other than those specified in the agreement, excluding use for audit purposes.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>The AI model is owned by the vendor unless otherwise agreed in writing.</t>
+          <t>Processor is prohibited from using data for purposes other than those specified in the agreement, excluding use for any internal operations.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>The AI model is owned by the vendor and cannot be transferred to the client.</t>
+          <t>Processor is authorized to use data for any purpose without restriction.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Professional Services IP Rights</t>
+          <t>Security Compliance</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>All IP developed during the engagement is owned by the client.</t>
+          <t>Compliance with ISO 27001 and SOC 2 standards is required.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>All IP developed during the engagement is owned by the client unless otherwise agreed in writing.</t>
+          <t>Compliance with ISO 27001 or SOC 2 standards is required.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>All IP developed during the engagement is owned by the client, with appropriate attribution.</t>
+          <t>Compliance with at least one of ISO 27001 or SOC 2 standards is required.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>All IP developed during the engagement is owned by the client, with a right of use granted to the vendor.</t>
+          <t>Compliance with a recognized information security standard is required.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>The vendor retains ownership of all IP developed during the engagement.</t>
+          <t>Compliance with no specific security standards is required.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>The vendor retains ownership of all IP and the client has no rights.</t>
+          <t>Compliance with no security standards is required.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Enterprise Software Security Compliance</t>
+          <t>IP Assignment</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>The software must comply with all applicable security standards and certifications.</t>
+          <t>All IP developed during the engagement is assigned to the client.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>The software must comply with the most relevant security standards and certifications.</t>
+          <t>All IP developed during the engagement is assigned to the client, excluding IP developed by third parties.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>The software must comply with a minimum set of security standards and certifications.</t>
+          <t>All IP developed during the engagement is assigned to the client, excluding IP developed using pre-existing client IP.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>The software must comply with a baseline set of security standards and certifications.</t>
+          <t>All IP developed during the engagement is assigned to the client, excluding IP developed using open-source software.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>The software is not required to comply with any security standards or certifications.</t>
+          <t>All IP developed during the engagement is assigned to the client, excluding IP developed using any third-party IP.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>The software may be used without any security compliance requirements.</t>
+          <t>No IP is assigned to the client.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Procurement Contract Term Limits</t>
+          <t>Procurement Terms</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>The contract term is limited to a maximum of three years with automatic renewal options.</t>
+          <t>Supplier agrees to provide services at the lowest commercially reasonable rate.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>The contract term is limited to a maximum of two years with automatic renewal options.</t>
+          <t>Supplier agrees to provide services at a rate not exceeding the market rate.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>The contract term is limited to a maximum of one year with automatic renewal options.</t>
+          <t>Supplier agrees to provide services at a rate not exceeding the average industry rate.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>The contract term is limited to a maximum of one year with no automatic renewal options.</t>
+          <t>Supplier agrees to provide services at a rate not exceeding the supplier's standard rate.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>The contract term is not limited and may be extended indefinitely.</t>
+          <t>Supplier agrees to provide services at a rate not exceeding the supplier's standard rate plus a 10% markup.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>The contract has no term limit and may be extended indefinitely without notice.</t>
+          <t>Supplier agrees to provide services at a rate not exceeding the supplier's standard rate plus a 30% markup.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Data Processing Agreement Sub-Processing</t>
+          <t>AI Vendor Terms</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>The vendor must obtain prior written consent from the client before engaging any sub-processors.</t>
+          <t>Vendor is prohibited from using customer data for training AI models without explicit consent.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>The vendor must notify the client in writing before engaging any sub-processors.</t>
+          <t>Vendor is prohibited from using customer data for training AI models without explicit consent, excluding data used for model improvement.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>The vendor may engage sub-processors with the client's approval.</t>
+          <t>Vendor is prohibited from using customer data for training AI models without explicit consent, excluding data used for performance analytics.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>The vendor may engage sub-processors with the client's consent.</t>
+          <t>Vendor is prohibited from using customer data for training AI models without explicit consent, excluding data used for system optimization.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>The vendor may engage sub-processors without the client's consent.</t>
+          <t>Vendor is prohibited from using customer data for training AI models without explicit consent, excluding data used for internal testing.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>The vendor is not required to obtain the client's consent for sub-processing.</t>
+          <t>Vendor is authorized to use customer data for training AI models without explicit consent.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>IP Assignment in SaaS Development</t>
+          <t>Professional Services Agreement</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>All IP developed during the engagement is assigned to the client upon payment of the final milestone.</t>
+          <t>Client retains ownership of all deliverables and intellectual property created during the engagement.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>All IP developed during the engagement is assigned to the client upon completion of the project.</t>
+          <t>Client retains ownership of all deliverables created during the engagement, excluding intellectual property developed by the vendor.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>All IP developed during the engagement is assigned to the client upon acceptance of deliverables.</t>
+          <t>Client retains ownership of all deliverables created during the engagement, excluding intellectual property developed using pre-existing client IP.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>All IP developed during the engagement is assigned to the client upon receipt of the final deliverable.</t>
+          <t>Client retains ownership of all deliverables created during the engagement, excluding intellectual property developed using open-source software.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>The vendor retains ownership of all IP developed during the engagement.</t>
+          <t>Client retains ownership of all deliverables created during the engagement, excluding intellectual property developed using any third-party IP.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>The vendor retains ownership of all IP and the client has no rights.</t>
+          <t>Client does not retain ownership of any deliverables or intellectual property.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AI Vendor Data Usage Restrictions</t>
+          <t>Enterprise Software Licensing</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>The vendor may use the client's data solely for the purpose of providing the AI service.</t>
+          <t>License grants access to the software for all users within the organization.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>The vendor may use the client's data solely for the purpose of developing and improving the AI service.</t>
+          <t>License grants access to the software for all users within the organization, excluding third-party contractors.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>The vendor may use the client's data for the purpose of providing and improving the AI service.</t>
+          <t>License grants access to the software for all users within the organization, excluding remote employees.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>The vendor may use the client's data for the purpose of providing the AI service.</t>
+          <t>License grants access to the software for all users within the organization, excluding seasonal employees.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>The vendor may use the client's data for any purpose.</t>
+          <t>License grants access to the software for all users within the organization, excluding employees on leave.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>The vendor may use the client's data for any purpose without restriction.</t>
+          <t>License grants access to the software for no users.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Professional Services Termination Rights</t>
+          <t>Data Breach Notification</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>The client may terminate the engagement with 30 days' written notice.</t>
+          <t>Notification of a data breach must occur within 72 hours of discovery.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>The client may terminate the engagement with 15 days' written notice.</t>
+          <t>Notification of a data breach must occur within 7 days of discovery.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>The client may terminate the engagement with 7 days' written notice.</t>
+          <t>Notification of a data breach must occur within 14 days of discovery.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>The client may terminate the engagement with 3 days' written notice.</t>
+          <t>Notification of a data breach must occur within 30 days of discovery.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>The client may terminate the engagement with no notice.</t>
+          <t>Notification of a data breach must occur within 60 days of discovery.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>The client may not terminate the engagement under any circumstances.</t>
+          <t>Notification of a data breach is not required.</t>
         </is>
       </c>
     </row>
@@ -1571,735 +1571,735 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Both parties agree to mutual non-disclosure with defined scope and duration.</t>
+          <t>Both parties agree to mutual non-disclosure of all confidential information exchanged during negotiations.</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>One party agrees to non-disclosure with limited scope.</t>
+          <t>Confidentiality is limited to information disclosed by the other party.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>One party agrees to non-disclosure with no defined duration.</t>
+          <t>Disclosure is permitted if necessary for legal compliance.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>One party agrees to non-disclosure with no defined scope or duration.</t>
+          <t>Non-disclosure is limited to information related to the subject matter of the agreement.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Non-disclosure is required only for the disclosing party.</t>
+          <t>Confidentiality extends to all information, including internal business strategies.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>No non-disclosure agreement is acceptable.</t>
+          <t>Disclosure of all information is permitted without restriction.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SaaS Data Processing</t>
+          <t>SaaS Service Level Agreement</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Data is processed in compliance with GDPR and CCPA standards.</t>
+          <t>Service availability is guaranteed at 99.9% uptime with monthly service credits for downtime.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Data is processed in compliance with GDPR standards.</t>
+          <t>Service availability is guaranteed at 99% uptime with monthly service credits for downtime.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Data is processed in compliance with basic data protection principles.</t>
+          <t>Service availability is guaranteed at 95% uptime with no service credits.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Data processing is not defined.</t>
+          <t>Service availability is guaranteed at 90% uptime with no service credits.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Data is processed without any legal compliance requirements.</t>
+          <t>Service availability is guaranteed at 100% uptime with no service credits.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Data processing is prohibited without explicit user consent.</t>
+          <t>No service level guarantees are provided.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>AI Vendor Terms</t>
+          <t>Data Processing Agreement</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Vendor agrees to audit access and transparency on model training data.</t>
+          <t>Data processing is limited to the purposes specified in the agreement and compliance with GDPR and CCPA.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Vendor agrees to audit access but not transparency on model training data.</t>
+          <t>Data processing is limited to the purposes specified in the agreement and compliance with GDPR.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Vendor agrees to limited audit access.</t>
+          <t>Data processing is limited to the purposes specified in the agreement and compliance with GDPR or CCPA.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Vendor does not agree to any audit access.</t>
+          <t>Data processing is limited to the purposes specified in the agreement.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Vendor refuses to allow any form of audit or transparency.</t>
+          <t>Data processing is permitted for any purpose without restriction.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Vendor denies access to model training data altogether.</t>
+          <t>No data processing restrictions are applied.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Professional Services IP Ownership</t>
+          <t>Security Compliance Requirements</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>All work product is owned by the client with full IP rights.</t>
+          <t>The vendor must comply with ISO 27001 and SOC 2 standards and provide annual audit reports.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>All work product is owned by the client with limited IP rights.</t>
+          <t>The vendor must comply with SOC 2 standards and provide annual audit reports.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Work product is owned by the client with a right of first refusal.</t>
+          <t>The vendor must comply with ISO 27001 standards and provide annual audit reports.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Work product is owned by the vendor with limited client rights.</t>
+          <t>The vendor must provide annual audit reports.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Work product is owned by the vendor with no client rights.</t>
+          <t>The vendor must comply with ISO 27001 and SOC 2 standards without audit reports.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Client has no rights to any work product.</t>
+          <t>No security compliance requirements are imposed.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Enterprise Software Security Compliance</t>
+          <t>IP Ownership in AI Development</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Vendor complies with ISO 27001 and SOC 2 standards.</t>
+          <t>All intellectual property developed during the project is owned by the client with full rights to commercialize.</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Vendor complies with SOC 2 standards.</t>
+          <t>All intellectual property developed during the project is owned by the client with limited rights to commercialize.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Vendor complies with basic security best practices.</t>
+          <t>All intellectual property developed during the project is owned by the client with rights to use for internal purposes.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Vendor has no defined security compliance standards.</t>
+          <t>Intellectual property ownership is shared 50-50 between the client and vendor.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Vendor does not comply with any security standards.</t>
+          <t>Intellectual property ownership is retained by the vendor with limited licensing rights.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Vendor denies responsibility for security compliance.</t>
+          <t>No intellectual property rights are transferred to the client.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Procurement Contract Term Limits</t>
+          <t>Procurement Contract Terms</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Contract term is limited to 3 years with automatic renewal option.</t>
+          <t>The vendor agrees to deliver the goods or services within 30 days of contract execution with a 5% penalty for late delivery.</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Contract term is limited to 3 years with no automatic renewal option.</t>
+          <t>The vendor agrees to deliver the goods or services within 45 days of contract execution with a 5% penalty for late delivery.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Contract term is limited to 1 year with automatic renewal option.</t>
+          <t>The vendor agrees to deliver the goods or services within 60 days of contract execution with no penalty for late delivery.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Contract term is unlimited with no automatic renewal option.</t>
+          <t>The vendor agrees to deliver the goods or services within 90 days of contract execution with no penalty for late delivery.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Contract term is unlimited with no renewal option.</t>
+          <t>The vendor agrees to deliver the goods or services within 120 days of contract execution with no penalty for late delivery.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Contract term is unlimited with no termination rights.</t>
+          <t>No delivery timelines or penalties are specified.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Data Breach Notification Requirements</t>
+          <t>AI Vendor Terms for Model Access</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Breach must be notified within 72 hours and reported to regulatory bodies.</t>
+          <t>The client is granted full access to the AI model for training and evaluation purposes with no restrictions.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Breach must be notified within 7 days and reported to regulatory bodies.</t>
+          <t>The client is granted limited access to the AI model for training purposes only.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Breach must be notified within 7 days with no regulatory reporting.</t>
+          <t>The client is granted access to the AI model for evaluation purposes only.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Breach notification is not required.</t>
+          <t>The client is granted access to the AI model with usage restrictions.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Breach notification is required only for the vendor.</t>
+          <t>The client is granted access to the AI model with no usage restrictions.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Breach notification is not required for either party.</t>
+          <t>No access to the AI model is granted.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>IP Assignment in Software Development</t>
+          <t>Professional Services Scope of Work</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>All IP is assigned to the client with no vendor rights.</t>
+          <t>The vendor agrees to provide all services as defined in the detailed scope of work with no additional charges for scope changes.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>All IP is assigned to the client with limited vendor rights.</t>
+          <t>The vendor agrees to provide all services as defined in the detailed scope of work with limited additional charges for scope changes.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>All IP is assigned to the client with a right of first refusal.</t>
+          <t>The vendor agrees to provide all services as defined in the detailed scope of work with additional charges for scope changes.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>IP is shared with vendor and client.</t>
+          <t>The vendor agrees to provide all services as defined in the scope of work with no additional charges for minor scope changes.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>IP is owned by the vendor with no client rights.</t>
+          <t>The vendor agrees to provide all services as defined in the scope of work with no additional charges for any scope changes.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>IP is not assigned to the client.</t>
+          <t>No scope of work is defined and no additional charges are permitted.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Security Incident Response Plan</t>
+          <t>Enterprise Software Licensing Model</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Vendor provides a detailed incident response plan with defined roles and timelines.</t>
+          <t>The client is granted a perpetual license with no usage limits and annual maintenance fees at 15% of the initial license cost.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Vendor provides a detailed incident response plan with defined roles.</t>
+          <t>The client is granted a perpetual license with no usage limits and annual maintenance fees at 20% of the initial license cost.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Vendor provides a basic incident response plan.</t>
+          <t>The client is granted a perpetual license with usage limits and annual maintenance fees at 25% of the initial license cost.</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Vendor provides no incident response plan.</t>
+          <t>The client is granted a perpetual license with annual maintenance fees at 30% of the initial license cost.</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Vendor denies responsibility for incident response.</t>
+          <t>The client is granted a perpetual license with no maintenance fees.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Vendor refuses to provide any incident response plan.</t>
+          <t>No perpetual license is granted and no maintenance fees are required.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cloud Data Residency Compliance</t>
+          <t>Data Privacy and Consent Clause</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Data is stored in EU data centers with compliance certifications.</t>
+          <t>The vendor must obtain explicit consent from all data subjects before processing their personal data.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Data is stored in EU data centers without compliance certifications.</t>
+          <t>The vendor must obtain implicit consent from all data subjects before processing their personal data.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Data is stored in data centers with no defined location.</t>
+          <t>The vendor must obtain consent from data subjects in certain cases.</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Data is stored in data centers with no defined compliance requirements.</t>
+          <t>The vendor must obtain consent from data subjects where required by law.</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Data is stored in data centers outside EU with no compliance requirements.</t>
+          <t>The vendor must obtain consent from data subjects in all cases.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Data storage location is not defined.</t>
+          <t>No consent is required from data subjects.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>NDA Mutual Non-Disclosure</t>
+          <t>NDA Mutual Nondisclosure</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Both parties agree to mutual non-disclosure of all confidential information exchanged during negotiations.</t>
+          <t>Both parties agree to mutual nondisclosure with equal confidentiality obligations and defined disclosure periods.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Confidentiality applies only to the disclosing party's information.</t>
+          <t>One party agrees to nondisclosure while the other may disclose limited information under specific conditions.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Non-disclosure is limited to information provided in written form.</t>
+          <t>One party agrees to nondisclosure with the other party having limited disclosure rights under agreed terms.</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Non-disclosure is limited to information exchanged during the term of the agreement.</t>
+          <t>One party agrees to nondisclosure with no defined disclosure period or scope.</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Confidentiality does not apply to information shared by the other party.</t>
+          <t>Confidentiality obligations are not reciprocal or include exceptions for public information.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Disclosure of all information is permitted without restriction.</t>
+          <t>No confidentiality obligations are agreed upon by either party.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SaaS Data Processing</t>
+          <t>SaaS Service Level Agreement</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Data processing is governed by EU GDPR and other applicable data protection laws.</t>
+          <t>Service level objectives are defined with clear performance metrics and escalation procedures.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Data processing complies with the data controller's local laws.</t>
+          <t>Service level objectives are defined with less detailed performance metrics and limited escalation procedures.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Data processing is subject to the processor's local data laws.</t>
+          <t>Service level objectives are defined with general performance metrics and no defined escalation procedures.</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Data processing is governed by the jurisdiction of the service provider.</t>
+          <t>Service level objectives are defined without specific metrics or escalation procedures.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Data processing is not subject to any data protection laws.</t>
+          <t>No defined service level objectives or performance metrics are agreed upon.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Data processing is unrestricted and not subject to any legal compliance.</t>
+          <t>No service level agreement is agreed upon.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AI Vendor Terms Model Transparency</t>
+          <t>Data Processing Agreement</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Vendor provides full transparency on AI model training data and algorithms.</t>
+          <t>Data processing is governed by strict compliance with applicable data protection laws and regular audits.</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Vendor provides limited transparency on AI model training data.</t>
+          <t>Data processing is governed by compliance with applicable data protection laws without regular audits.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Vendor provides transparency on AI model training data upon request.</t>
+          <t>Data processing is governed by compliance with applicable data protection laws with limited audit rights.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Vendor provides transparency on AI model training data in summary form.</t>
+          <t>Data processing is governed by compliance with applicable data protection laws with no audit rights.</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Vendor does not provide any transparency on AI model training data.</t>
+          <t>No compliance with data protection laws is required.</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Vendor refuses to disclose any information about AI model training data.</t>
+          <t>No data protection requirements are agreed upon.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Professional Services Termination Notice</t>
+          <t>Security Compliance Requirements</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Termination notice period is 30 days with cause.</t>
+          <t>All security requirements are defined with third-party audits and regular compliance checks.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Termination notice period is 15 days with cause.</t>
+          <t>All security requirements are defined with third-party audits but no regular compliance checks.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Termination notice period is 30 days without cause.</t>
+          <t>All security requirements are defined with limited audit rights and no regular compliance checks.</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Termination notice period is 7 days with cause.</t>
+          <t>All security requirements are defined without third-party audits or compliance checks.</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Termination notice period is zero days with cause.</t>
+          <t>No defined security requirements or audit processes are agreed upon.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Termination is not subject to any notice period.</t>
+          <t>No security compliance requirements are agreed upon.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Enterprise Software Data Residency</t>
+          <t>IP Ownership and Licensing</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Data is stored and processed in the customer's country of residence.</t>
+          <t>All intellectual property is owned by the company with full licensing rights and no restrictions.</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Data is stored and processed in the vendor's country of residence.</t>
+          <t>All intellectual property is owned by the company with limited licensing rights and restrictions.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Data is stored and processed in the country with the lowest regulatory burden.</t>
+          <t>All intellectual property is owned by the company with no defined licensing rights or restrictions.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Data is stored and processed in the country where the service is hosted.</t>
+          <t>All intellectual property is subject to third-party ownership with limited licensing rights.</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Data is stored and processed in a third-party country without restriction.</t>
+          <t>No defined IP ownership or licensing rights are agreed upon.</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Data is stored and processed in a country with no data residency requirements.</t>
+          <t>No IP ownership or licensing rights are agreed upon.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IP Assignment in Procurement Agreements</t>
+          <t>Procurement Contract Terms</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>All IP developed during the procurement is assigned to the customer.</t>
+          <t>Procurement terms include fixed pricing, defined deliverables, and clear performance metrics.</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>IP developed during the procurement is owned by the vendor with a non-exclusive license to the customer.</t>
+          <t>Procurement terms include fixed pricing with limited deliverables and performance metrics.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>IP developed during the procurement is shared jointly with the customer.</t>
+          <t>Procurement terms include fixed pricing with no defined deliverables or performance metrics.</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>IP developed during the procurement is owned by the vendor with a royalty-free license to the customer.</t>
+          <t>Procurement terms include variable pricing with no defined deliverables or performance metrics.</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>IP developed during the procurement is not assigned or licensed to the customer.</t>
+          <t>No defined pricing, deliverables, or performance metrics are agreed upon.</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>IP developed during the procurement is exclusively owned by the vendor with no rights granted to the customer.</t>
+          <t>No procurement terms are agreed upon.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Security Incident Response Timeline</t>
+          <t>AI Vendor Terms and Usage</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Vendor must notify customer of security incidents within 24 hours.</t>
+          <t>AI vendor terms include usage limits, data ownership, and strict compliance with ethical guidelines.</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Vendor must notify customer of security incidents within 48 hours.</t>
+          <t>AI vendor terms include usage limits and data ownership with limited compliance with ethical guidelines.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Vendor must notify customer of security incidents within 72 hours.</t>
+          <t>AI vendor terms include usage limits with no defined data ownership or compliance with ethical guidelines.</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Vendor must notify customer of security incidents within 5 business days.</t>
+          <t>AI vendor terms include no defined usage limits, data ownership, or ethical guidelines.</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Vendor is not required to notify the customer of security incidents.</t>
+          <t>No defined AI vendor terms or ethical guidelines are agreed upon.</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Vendor is not required to notify the customer of any security incidents.</t>
+          <t>No AI vendor terms are agreed upon.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Data Breach Notification Requirements</t>
+          <t>Professional Services Scope and Payment</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Vendor must notify customer of data breaches within 72 hours of discovery.</t>
+          <t>Scope and payment terms are defined with clear deliverables, timelines, and payment milestones.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Vendor must notify customer of data breaches within 14 days of discovery.</t>
+          <t>Scope and payment terms are defined with clear deliverables and timelines but no payment milestones.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Vendor must notify customer of data breaches within 30 days of discovery.</t>
+          <t>Scope and payment terms are defined with limited deliverables and timelines but no payment milestones.</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Vendor must notify customer of data breaches within 10 business days of discovery.</t>
+          <t>Scope and payment terms are defined with no deliverables, timelines, or payment milestones.</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Vendor is not required to notify the customer of data breaches.</t>
+          <t>No defined scope, payment terms, or deliverables are agreed upon.</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Vendor is not required to notify the customer of any data breaches.</t>
+          <t>No professional services agreement is agreed upon.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>NDA Exclusions for Public Information</t>
+          <t>Enterprise Software Licensing</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Exclusions apply only to information that is publicly available.</t>
+          <t>Licensing terms include per-user pricing, usage limits, and regular audit rights.</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Exclusions apply to information that is not confidential.</t>
+          <t>Licensing terms include per-user pricing with limited usage limits and audit rights.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Exclusions apply to information that is not sensitive.</t>
+          <t>Licensing terms include per-user pricing with no defined usage limits or audit rights.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Exclusions apply to information that is not protected by law.</t>
+          <t>Licensing terms include no defined pricing, usage limits, or audit rights.</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Exclusions apply to all information regardless of confidentiality.</t>
+          <t>No defined licensing terms or audit rights are agreed upon.</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Exclusions apply to all information and no information is protected.</t>
+          <t>No licensing terms are agreed upon.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Vendor Audit Rights in SaaS Agreements</t>
+          <t>Data Transfer and Storage Agreements</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Vendor grants the customer the right to audit the service provider's data processing activities.</t>
+          <t>Data transfer and storage are governed by strict security standards and defined data residency requirements.</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Vendor grants the customer the right to audit the service provider's data processing activities upon request.</t>
+          <t>Data transfer and storage are governed by security standards with limited data residency requirements.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Vendor grants the customer the right to audit the service provider's data processing activities annually.</t>
+          <t>Data transfer and storage are governed by security standards with no defined data residency requirements.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Vendor grants the customer the right to audit the service provider's data processing activities semi-annually.</t>
+          <t>Data transfer and storage are governed by no defined security standards or data residency requirements.</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Vendor does not grant the customer the right to audit data processing activities.</t>
+          <t>No defined security standards or data residency requirements are agreed upon.</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Vendor refuses to allow any audits of data processing activities.</t>
+          <t>No data transfer or storage agreement is agreed upon.</t>
         </is>
       </c>
     </row>

</xml_diff>